<commit_message>
Update P&L with new fFacial data
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/fFacial.xlsx
+++ b/fFacial.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{D9D2D1F5-F5B2-413B-9EF5-9E3621390E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90B5B624-27A4-4C2A-B0BD-4F7676135491}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{D9D2D1F5-F5B2-413B-9EF5-9E3621390E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09F02CE2-91BA-475A-A387-1008604376A0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{87DA37B0-848D-436B-BEE1-46F60B206BED}"/>
+    <workbookView xWindow="-28920" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{87DA37B0-848D-436B-BEE1-46F60B206BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="72">
   <si>
     <t>fac-16</t>
   </si>
@@ -231,6 +231,30 @@
   </si>
   <si>
     <t>2026.04.01-CAMBR2-9</t>
+  </si>
+  <si>
+    <t>2026.01.21-CAMCA4-3</t>
+  </si>
+  <si>
+    <t>2026.01.24-CAMCA4-4</t>
+  </si>
+  <si>
+    <t>2026.01.29-CAMBR2-1</t>
+  </si>
+  <si>
+    <t>2026.02.01-CAMCA4-5</t>
+  </si>
+  <si>
+    <t>2026.02.15-CAMCA4-Quartas</t>
+  </si>
+  <si>
+    <t>2026.02.25-CAMLI5-2° FASE</t>
+  </si>
+  <si>
+    <t>2026.02.28-CAMCA4-SEMIS - TR</t>
+  </si>
+  <si>
+    <t>2026.04.12-CAMBR2-11</t>
   </si>
 </sst>
 </file>
@@ -624,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262C255-C934-4E6E-8069-0C0204B67DBD}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.54296875" style="3" bestFit="1" customWidth="1"/>
@@ -1388,6 +1412,94 @@
         <v>0</v>
       </c>
     </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>65</v>
+      </c>
+      <c r="B69" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>66</v>
+      </c>
+      <c r="B70" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>67</v>
+      </c>
+      <c r="B71" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>68</v>
+      </c>
+      <c r="B72" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>69</v>
+      </c>
+      <c r="B73" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>70</v>
+      </c>
+      <c r="B74" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75" s="5">
+        <v>-30800</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1" xr:uid="{6262C255-C934-4E6E-8069-0C0204B67DBD}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C48">

</xml_diff>